<commit_message>
Update Basket 1 to 5M PVD rollover at 3.5% and Basket 3 to 6.5M bonds
</commit_message>
<xml_diff>
--- a/Retirement_Plan_25M.xlsx
+++ b/Retirement_Plan_25M.xlsx
@@ -1795,7 +1795,7 @@
         <v>11500</v>
       </c>
       <c r="K23" s="15" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L23" s="9">
         <f>SUM(G23:K23)</f>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="P23" s="19" t="inlineStr">
         <is>
-          <t>สับ PVD+RMF เข้าตราสารหนี้ | ฝากพิเศษ สอ. 10k/ด. | บำนาญ 85/5 (ปี 3/5)</t>
+          <t>สับ PVD+RMF เข้าตราสารหนี้ | บำนาญ 85/5 (ปี 3/5)</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
         <v>12500</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L24" s="9">
         <f>SUM(G24:K24)</f>
@@ -1869,7 +1869,7 @@
       </c>
       <c r="P24" s="12" t="inlineStr">
         <is>
-          <t>บำนาญ 85/5 (ปี 4/5) | ปรับเบี้ยสุขภาพช่วง 56-60 | ฝากพิเศษ 10k/ด.</t>
+          <t>บำนาญ 85/5 (ปี 4/5) | ปรับเบี้ยสุขภาพช่วง 56-60</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
         <v>12500</v>
       </c>
       <c r="K25" s="22" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L25" s="9">
         <f>SUM(G25:K25)</f>
@@ -1960,7 +1960,7 @@
         <v>9167</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L26" s="9">
         <f>SUM(G26:K26)</f>
@@ -2015,7 +2015,7 @@
         <v>9167</v>
       </c>
       <c r="K27" s="15" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L27" s="9">
         <f>SUM(G27:K27)</f>
@@ -2034,7 +2034,7 @@
       </c>
       <c r="P27" s="19" t="inlineStr">
         <is>
-          <t>เตรียมความพร้อมก่อนเกษียณ 1 ปี</t>
+          <t>เตรียมความพร้อมก่อนเกษียณ 1 ปี (วางแผนโยก PVD เข้า สอ. ภายใน 60 วัน)</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
         <v>9167</v>
       </c>
       <c r="K28" s="22" t="n">
-        <v>10000</v>
+        <v>0</v>
       </c>
       <c r="L28" s="9">
         <f>SUM(G28:K28)</f>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="P28" s="26" t="inlineStr">
         <is>
-          <t>ปีสุดท้าย: ส่งบำนาญเดิมงวดสุดท้าย + รับเงินชดเชยเกษียณ 400 วัน 1.312M</t>
+          <t>ปีสุดท้าย: ส่งบำนาญเดิมงวดสุดท้าย + รับเงินชดเชยเกษียณ 400 วัน 1.312M + โยก PVD 5M ฝากพิเศษเกษียณสุข</t>
         </is>
       </c>
     </row>
@@ -2324,14 +2324,14 @@
         </is>
       </c>
       <c r="D6" s="35" t="n">
-        <v>6000000</v>
+        <v>5000000</v>
       </c>
       <c r="E6" s="36">
         <f>D6/D12</f>
         <v/>
       </c>
       <c r="F6" s="37" t="n">
-        <v>0.0375</v>
+        <v>0.035</v>
       </c>
       <c r="G6" s="6">
         <f>ROUND(D6*F6, 0)</f>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="I6" s="38" t="inlineStr">
         <is>
-          <t>เครื่องจักรผลิตดอกเบี้ยหลัก ปลอดภัยสูง (ปลอดภาษี)</t>
+          <t>โยกจาก PVD สูงสุด 5 ล้านบาท ภายใน 60 วัน (ปลอดภาษี)</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2390,7 @@
         </is>
       </c>
       <c r="D8" s="35" t="n">
-        <v>5500000</v>
+        <v>6500000</v>
       </c>
       <c r="E8" s="36">
         <f>D8/D12</f>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="I8" s="38" t="inlineStr">
         <is>
-          <t>ล็อกผลตอบแทนระยะยาว ไร้ความเสี่ยงผิดนัด (หลังหักภาษี 15%)</t>
+          <t>ล็อกผลตอบแทนระยะยาว ไร้ความเสี่ยงผิดนัด (เพิ่ม 1 ล้าน) (หลังหักภาษี 15%)</t>
         </is>
       </c>
     </row>
@@ -2541,7 +2541,7 @@
       </c>
       <c r="I12" s="27" t="inlineStr">
         <is>
-          <t>ผลิตกระแสเงินสดเฉลี่ย 56,258 บ./เดือน (รวมท่อคุณแม่ 15,000 บ./ด.)</t>
+          <t>ผลิตกระแสเงินสดเฉลี่ย 54,004 บ./เดือน (รวมท่อคุณแม่ 15,000 บ./ด.)</t>
         </is>
       </c>
     </row>
@@ -2618,7 +2618,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>ท่อที่ 1 คุณแม่ (15,000 บ./ด.) | ท่อที่ 2 ส่วนตัวคุณ (52,291 บ./ด.) พร้อมแผน Drawdown ปลอดภัย</t>
+          <t>ท่อที่ 1 คุณแม่ (15,000 บ./ด.) | ท่อที่ 2 ส่วนตัวคุณ (50,038 บ./ด.) พร้อมแผน Drawdown ปลอดภัย</t>
         </is>
       </c>
     </row>
@@ -2691,10 +2691,10 @@
         </is>
       </c>
       <c r="D8" s="52" t="n">
-        <v>495100</v>
+        <v>468050</v>
       </c>
       <c r="E8" s="40" t="n">
-        <v>41258</v>
+        <v>39004</v>
       </c>
       <c r="F8" s="43" t="inlineStr">
         <is>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="F12" s="53" t="inlineStr">
         <is>
-          <t>เงินสดรับส่วนตัว 52,291 บาท/เดือน (627,500 บ./ปี)</t>
+          <t>เงินสดรับส่วนตัว 50,038 บาท/เดือน (600,450 บ./ปี)</t>
         </is>
       </c>
     </row>
@@ -2838,7 +2838,7 @@
       </c>
       <c r="C16" s="43" t="inlineStr">
         <is>
-          <t>66.9% ของกระแสเงินสดรับส่วนตัว</t>
+          <t>69.9% ของกระแสเงินสดรับส่วนตัว</t>
         </is>
       </c>
       <c r="D16" s="52" t="n">
@@ -2861,14 +2861,14 @@
       </c>
       <c r="C17" s="43" t="inlineStr">
         <is>
-          <t>33.1% ของกระแสเงินสดรับส่วนตัว</t>
+          <t>30.1% ของกระแสเงินสดรับส่วนตัว</t>
         </is>
       </c>
       <c r="D17" s="52" t="n">
-        <v>207500</v>
+        <v>180450</v>
       </c>
       <c r="E17" s="40" t="n">
-        <v>17291</v>
+        <v>15038</v>
       </c>
       <c r="F17" s="43" t="inlineStr">
         <is>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="E22" s="38" t="inlineStr">
         <is>
-          <t>ใช้จ่ายเฉพาะดอกเบี้ยและบำนาญ 52,291 บ./ด. แบ่ง 500k จากตะกร้า 6 ไว้เป็นกองทุนฉุกเฉินคุณแม่</t>
+          <t>ใช้จ่ายเฉพาะดอกเบี้ยและบำนาญ 50,038 บ./ด. แบ่ง 500k จากตะกร้า 6 ไว้เป็นกองทุนฉุกเฉินคุณแม่</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="E24" s="38" t="inlineStr">
         <is>
-          <t>คุณแม่อายุ 98 ปี หุ้น สอ. 4M ปลดล็อกกลับมาเป็นสภาพคล่องส่วนตัว ไถ่ถอน MMF 4M และพันธบัตร 5.5M ตามลำดับ โดยคงเงินฝากพิเศษ 6M และทองคำ 5 บาทไว้ท้ายสุด</t>
+          <t>คุณแม่อายุ 98 ปี หุ้น สอ. 4M ปลดล็อกกลับมาเป็นสภาพคล่องส่วนตัว ไถ่ถอน MMF 4M และพันธบัตร 6.5M ตามลำดับ โดยคงเงินฝากพิเศษ 5M และทองคำ 5 บาทไว้ท้ายสุด</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove unused 'coop special deposit' column across dashboard, Excel, and CSV
</commit_message>
<xml_diff>
--- a/Retirement_Plan_25M.xlsx
+++ b/Retirement_Plan_25M.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:P37"/>
+  <dimension ref="B2:O37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -729,12 +729,11 @@
     <col width="18" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -799,30 +798,25 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>ฝากพิเศษ สอ. (บ./ด.)</t>
+          <t>รวมหักเงินเดือนประจำ</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>รวมหักเงินเดือนประจำ</t>
+          <t>บำนาญใหม่ (โบนัส)</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
         <is>
-          <t>บำนาญใหม่ (โบนัส)</t>
+          <t>รวมจ่ายทั้งปี (บาท)</t>
         </is>
       </c>
       <c r="N5" s="3" t="inlineStr">
         <is>
-          <t>รวมจ่ายทั้งปี (บาท)</t>
+          <t>เงินเหลือใช้สุทธิ/ปี</t>
         </is>
       </c>
       <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>เงินเหลือใช้สุทธิ/ปี</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>หมุดหมายสำคัญ / Strategic Action</t>
         </is>
@@ -859,25 +853,22 @@
       <c r="J6" s="6" t="n">
         <v>9583</v>
       </c>
-      <c r="K6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="9">
-        <f>SUM(G6:K6)</f>
-        <v/>
-      </c>
-      <c r="M6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="10">
-        <f>L6*12+M6</f>
-        <v/>
-      </c>
-      <c r="O6" s="11">
-        <f>F6-N6</f>
-        <v/>
-      </c>
-      <c r="P6" s="12" t="inlineStr">
+      <c r="K6" s="9">
+        <f>SUM(G6:J6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="10">
+        <f>K6*12+L6</f>
+        <v/>
+      </c>
+      <c r="N6" s="11">
+        <f>F6-M6</f>
+        <v/>
+      </c>
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>เริ่มแผน: สอ. 20k/ด. ล็อกเป้า 4M, RMF 2k/ด., PVD 15%</t>
         </is>
@@ -914,25 +905,22 @@
       <c r="J7" s="15" t="n">
         <v>9583</v>
       </c>
-      <c r="K7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="9">
-        <f>SUM(G7:K7)</f>
-        <v/>
-      </c>
-      <c r="M7" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="10">
-        <f>L7*12+M7</f>
-        <v/>
-      </c>
-      <c r="O7" s="18">
-        <f>F7-N7</f>
-        <v/>
-      </c>
-      <c r="P7" s="19" t="inlineStr">
+      <c r="K7" s="9">
+        <f>SUM(G7:J7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="10">
+        <f>K7*12+L7</f>
+        <v/>
+      </c>
+      <c r="N7" s="18">
+        <f>F7-M7</f>
+        <v/>
+      </c>
+      <c r="O7" s="19" t="inlineStr">
         <is>
           <t>ฐานเงินเดือนโต 5% ต่อปี</t>
         </is>
@@ -969,25 +957,22 @@
       <c r="J8" s="6" t="n">
         <v>9583</v>
       </c>
-      <c r="K8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="9">
-        <f>SUM(G8:K8)</f>
-        <v/>
-      </c>
-      <c r="M8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" s="10">
-        <f>L8*12+M8</f>
-        <v/>
-      </c>
-      <c r="O8" s="11">
-        <f>F8-N8</f>
-        <v/>
-      </c>
-      <c r="P8" s="12" t="inlineStr">
+      <c r="K8" s="9">
+        <f>SUM(G8:J8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="10">
+        <f>K8*12+L8</f>
+        <v/>
+      </c>
+      <c r="N8" s="11">
+        <f>F8-M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="12" t="inlineStr">
         <is>
           <t>สะสมหุ้น สอ. ต่อเนื่อง</t>
         </is>
@@ -1024,25 +1009,22 @@
       <c r="J9" s="15" t="n">
         <v>10000</v>
       </c>
-      <c r="K9" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="9">
-        <f>SUM(G9:K9)</f>
-        <v/>
-      </c>
-      <c r="M9" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" s="10">
-        <f>L9*12+M9</f>
-        <v/>
-      </c>
-      <c r="O9" s="18">
-        <f>F9-N9</f>
-        <v/>
-      </c>
-      <c r="P9" s="19" t="inlineStr">
+      <c r="K9" s="9">
+        <f>SUM(G9:J9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="10">
+        <f>K9*12+L9</f>
+        <v/>
+      </c>
+      <c r="N9" s="18">
+        <f>F9-M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="19" t="inlineStr">
         <is>
           <t>ปรับเบี้ยประกันสุขภาพตามช่วงอายุ</t>
         </is>
@@ -1079,25 +1061,22 @@
       <c r="J10" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="K10" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" s="9">
-        <f>SUM(G10:K10)</f>
-        <v/>
-      </c>
-      <c r="M10" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="10">
-        <f>L10*12+M10</f>
-        <v/>
-      </c>
-      <c r="O10" s="25">
-        <f>F10-N10</f>
-        <v/>
-      </c>
-      <c r="P10" s="26" t="inlineStr">
+      <c r="K10" s="9">
+        <f>SUM(G10:J10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="10">
+        <f>K10*12+L10</f>
+        <v/>
+      </c>
+      <c r="N10" s="25">
+        <f>F10-M10</f>
+        <v/>
+      </c>
+      <c r="O10" s="26" t="inlineStr">
         <is>
           <t>ปีสุดท้ายที่ส่ง สอ.กฟผ. ครบเป้าหมายเงินต้น 4,000,000 บ.</t>
         </is>
@@ -1134,25 +1113,22 @@
       <c r="J11" s="22" t="n">
         <v>10000</v>
       </c>
-      <c r="K11" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="9">
-        <f>SUM(G11:K11)</f>
-        <v/>
-      </c>
-      <c r="M11" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="10">
-        <f>L11*12+M11</f>
-        <v/>
-      </c>
-      <c r="O11" s="25">
-        <f>F11-N11</f>
-        <v/>
-      </c>
-      <c r="P11" s="26" t="inlineStr">
+      <c r="K11" s="9">
+        <f>SUM(G11:J11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="10">
+        <f>K11*12+L11</f>
+        <v/>
+      </c>
+      <c r="N11" s="25">
+        <f>F11-M11</f>
+        <v/>
+      </c>
+      <c r="O11" s="26" t="inlineStr">
         <is>
           <t>หยุดส่ง สอ. (ปันผล 15k/ด. โอนให้แม่ 100%), เร่ง RMF เป็น 24k/ด.</t>
         </is>
@@ -1189,25 +1165,22 @@
       <c r="J12" s="6" t="n">
         <v>10000</v>
       </c>
-      <c r="K12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="9">
-        <f>SUM(G12:K12)</f>
-        <v/>
-      </c>
-      <c r="M12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="10">
-        <f>L12*12+M12</f>
-        <v/>
-      </c>
-      <c r="O12" s="11">
-        <f>F12-N12</f>
-        <v/>
-      </c>
-      <c r="P12" s="12" t="inlineStr">
+      <c r="K12" s="9">
+        <f>SUM(G12:J12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="10">
+        <f>K12*12+L12</f>
+        <v/>
+      </c>
+      <c r="N12" s="11">
+        <f>F12-M12</f>
+        <v/>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
         <is>
           <t>เร่งสปีดหุ้นโลกผ่าน PVD 15% + RMF 24k</t>
         </is>
@@ -1244,25 +1217,22 @@
       <c r="J13" s="15" t="n">
         <v>10000</v>
       </c>
-      <c r="K13" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="9">
-        <f>SUM(G13:K13)</f>
-        <v/>
-      </c>
-      <c r="M13" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="10">
-        <f>L13*12+M13</f>
-        <v/>
-      </c>
-      <c r="O13" s="18">
-        <f>F13-N13</f>
-        <v/>
-      </c>
-      <c r="P13" s="19" t="inlineStr">
+      <c r="K13" s="9">
+        <f>SUM(G13:J13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="10">
+        <f>K13*12+L13</f>
+        <v/>
+      </c>
+      <c r="N13" s="18">
+        <f>F13-M13</f>
+        <v/>
+      </c>
+      <c r="O13" s="19" t="inlineStr">
         <is>
           <t>ช่วงสะสมสินทรัพย์เติบโตสูง</t>
         </is>
@@ -1299,25 +1269,22 @@
       <c r="J14" s="6" t="n">
         <v>10667</v>
       </c>
-      <c r="K14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="9">
-        <f>SUM(G14:K14)</f>
-        <v/>
-      </c>
-      <c r="M14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="10">
-        <f>L14*12+M14</f>
-        <v/>
-      </c>
-      <c r="O14" s="11">
-        <f>F14-N14</f>
-        <v/>
-      </c>
-      <c r="P14" s="12" t="inlineStr">
+      <c r="K14" s="9">
+        <f>SUM(G14:J14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="10">
+        <f>K14*12+L14</f>
+        <v/>
+      </c>
+      <c r="N14" s="11">
+        <f>F14-M14</f>
+        <v/>
+      </c>
+      <c r="O14" s="12" t="inlineStr">
         <is>
           <t>ปรับเบี้ยประกันสุขภาพตามช่วงอายุ 46-50 ปี</t>
         </is>
@@ -1354,25 +1321,22 @@
       <c r="J15" s="15" t="n">
         <v>10667</v>
       </c>
-      <c r="K15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="9">
-        <f>SUM(G15:K15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="10">
-        <f>L15*12+M15</f>
-        <v/>
-      </c>
-      <c r="O15" s="18">
-        <f>F15-N15</f>
-        <v/>
-      </c>
-      <c r="P15" s="19" t="inlineStr">
+      <c r="K15" s="9">
+        <f>SUM(G15:J15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="10">
+        <f>K15*12+L15</f>
+        <v/>
+      </c>
+      <c r="N15" s="18">
+        <f>F15-M15</f>
+        <v/>
+      </c>
+      <c r="O15" s="19" t="inlineStr">
         <is>
           <t>เตรียมแตะเพดานเงินเดือน กฟผ.</t>
         </is>
@@ -1409,25 +1373,22 @@
       <c r="J16" s="22" t="n">
         <v>10667</v>
       </c>
-      <c r="K16" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="9">
-        <f>SUM(G16:K16)</f>
-        <v/>
-      </c>
-      <c r="M16" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="10">
-        <f>L16*12+M16</f>
-        <v/>
-      </c>
-      <c r="O16" s="25">
-        <f>F16-N16</f>
-        <v/>
-      </c>
-      <c r="P16" s="26" t="inlineStr">
+      <c r="K16" s="9">
+        <f>SUM(G16:J16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="10">
+        <f>K16*12+L16</f>
+        <v/>
+      </c>
+      <c r="N16" s="25">
+        <f>F16-M16</f>
+        <v/>
+      </c>
+      <c r="O16" s="26" t="inlineStr">
         <is>
           <t>ฐานเงินเดือนแตะเพดาน 100,000 บ. (PVD หักคงที่ 15,000 บ./ด.)</t>
         </is>
@@ -1464,25 +1425,22 @@
       <c r="J17" s="15" t="n">
         <v>10667</v>
       </c>
-      <c r="K17" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="9">
-        <f>SUM(G17:K17)</f>
-        <v/>
-      </c>
-      <c r="M17" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="10">
-        <f>L17*12+M17</f>
-        <v/>
-      </c>
-      <c r="O17" s="18">
-        <f>F17-N17</f>
-        <v/>
-      </c>
-      <c r="P17" s="19" t="inlineStr">
+      <c r="K17" s="9">
+        <f>SUM(G17:J17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="10">
+        <f>K17*12+L17</f>
+        <v/>
+      </c>
+      <c r="N17" s="18">
+        <f>F17-M17</f>
+        <v/>
+      </c>
+      <c r="O17" s="19" t="inlineStr">
         <is>
           <t>ปีสุดท้ายของการเร่ง RMF 24k/ด.</t>
         </is>
@@ -1519,25 +1477,22 @@
       <c r="J18" s="6" t="n">
         <v>10667</v>
       </c>
-      <c r="K18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="9">
-        <f>SUM(G18:K18)</f>
-        <v/>
-      </c>
-      <c r="M18" s="6" t="n">
+      <c r="K18" s="9">
+        <f>SUM(G18:J18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="6" t="n">
         <v>100000</v>
       </c>
-      <c r="N18" s="10">
-        <f>L18*12+M18</f>
-        <v/>
-      </c>
-      <c r="O18" s="11">
-        <f>F18-N18</f>
-        <v/>
-      </c>
-      <c r="P18" s="12" t="inlineStr">
+      <c r="M18" s="10">
+        <f>K18*12+L18</f>
+        <v/>
+      </c>
+      <c r="N18" s="11">
+        <f>F18-M18</f>
+        <v/>
+      </c>
+      <c r="O18" s="12" t="inlineStr">
         <is>
           <t>RMF ลดเหลือ 16k/ด. + ซื้อบำนาญใหม่ #3 จ่าย 100k/ปี จากโบนัส (ปี 1/5)</t>
         </is>
@@ -1574,25 +1529,22 @@
       <c r="J19" s="15" t="n">
         <v>11500</v>
       </c>
-      <c r="K19" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="9">
-        <f>SUM(G19:K19)</f>
-        <v/>
-      </c>
-      <c r="M19" s="15" t="n">
+      <c r="K19" s="9">
+        <f>SUM(G19:J19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="15" t="n">
         <v>100000</v>
       </c>
-      <c r="N19" s="10">
-        <f>L19*12+M19</f>
-        <v/>
-      </c>
-      <c r="O19" s="18">
-        <f>F19-N19</f>
-        <v/>
-      </c>
-      <c r="P19" s="19" t="inlineStr">
+      <c r="M19" s="10">
+        <f>K19*12+L19</f>
+        <v/>
+      </c>
+      <c r="N19" s="18">
+        <f>F19-M19</f>
+        <v/>
+      </c>
+      <c r="O19" s="19" t="inlineStr">
         <is>
           <t>บำนาญใหม่ #3 จ่าย 100k/ปี (ปี 2/5) | ปรับเบี้ยสุขภาพช่วง 51-55</t>
         </is>
@@ -1629,25 +1581,22 @@
       <c r="J20" s="6" t="n">
         <v>11500</v>
       </c>
-      <c r="K20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L20" s="9">
-        <f>SUM(G20:K20)</f>
-        <v/>
-      </c>
-      <c r="M20" s="6" t="n">
+      <c r="K20" s="9">
+        <f>SUM(G20:J20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="6" t="n">
         <v>100000</v>
       </c>
-      <c r="N20" s="10">
-        <f>L20*12+M20</f>
-        <v/>
-      </c>
-      <c r="O20" s="11">
-        <f>F20-N20</f>
-        <v/>
-      </c>
-      <c r="P20" s="12" t="inlineStr">
+      <c r="M20" s="10">
+        <f>K20*12+L20</f>
+        <v/>
+      </c>
+      <c r="N20" s="11">
+        <f>F20-M20</f>
+        <v/>
+      </c>
+      <c r="O20" s="12" t="inlineStr">
         <is>
           <t>บำนาญใหม่ #3 จ่าย 100k/ปี (ปี 3/5)</t>
         </is>
@@ -1684,25 +1633,22 @@
       <c r="J21" s="22" t="n">
         <v>11500</v>
       </c>
-      <c r="K21" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="9">
-        <f>SUM(G21:K21)</f>
-        <v/>
-      </c>
-      <c r="M21" s="22" t="n">
+      <c r="K21" s="9">
+        <f>SUM(G21:J21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="22" t="n">
         <v>200000</v>
       </c>
-      <c r="N21" s="10">
-        <f>L21*12+M21</f>
-        <v/>
-      </c>
-      <c r="O21" s="25">
-        <f>F21-N21</f>
-        <v/>
-      </c>
-      <c r="P21" s="26" t="inlineStr">
+      <c r="M21" s="10">
+        <f>K21*12+L21</f>
+        <v/>
+      </c>
+      <c r="N21" s="25">
+        <f>F21-M21</f>
+        <v/>
+      </c>
+      <c r="O21" s="26" t="inlineStr">
         <is>
           <t>ซื้อบำนาญ 85/5 เพิ่ม 100k/ปี (ปี 1/5) ซ้อนบำนาญ #3 (ปี 4/5) รวม 200k/ปี</t>
         </is>
@@ -1739,25 +1685,22 @@
       <c r="J22" s="6" t="n">
         <v>11500</v>
       </c>
-      <c r="K22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="9">
-        <f>SUM(G22:K22)</f>
-        <v/>
-      </c>
-      <c r="M22" s="6" t="n">
+      <c r="K22" s="9">
+        <f>SUM(G22:J22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="6" t="n">
         <v>200000</v>
       </c>
-      <c r="N22" s="10">
-        <f>L22*12+M22</f>
-        <v/>
-      </c>
-      <c r="O22" s="11">
-        <f>F22-N22</f>
-        <v/>
-      </c>
-      <c r="P22" s="12" t="inlineStr">
+      <c r="M22" s="10">
+        <f>K22*12+L22</f>
+        <v/>
+      </c>
+      <c r="N22" s="11">
+        <f>F22-M22</f>
+        <v/>
+      </c>
+      <c r="O22" s="12" t="inlineStr">
         <is>
           <t>บำนาญ 85/5 (ปี 2/5) + บำนาญ #3 (ปี 5/5 งวดสุดท้าย) รวม 200k/ปี</t>
         </is>
@@ -1794,25 +1737,22 @@
       <c r="J23" s="15" t="n">
         <v>11500</v>
       </c>
-      <c r="K23" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="9">
-        <f>SUM(G23:K23)</f>
-        <v/>
-      </c>
-      <c r="M23" s="15" t="n">
+      <c r="K23" s="9">
+        <f>SUM(G23:J23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="15" t="n">
         <v>100000</v>
       </c>
-      <c r="N23" s="10">
-        <f>L23*12+M23</f>
-        <v/>
-      </c>
-      <c r="O23" s="18">
-        <f>F23-N23</f>
-        <v/>
-      </c>
-      <c r="P23" s="19" t="inlineStr">
+      <c r="M23" s="10">
+        <f>K23*12+L23</f>
+        <v/>
+      </c>
+      <c r="N23" s="18">
+        <f>F23-M23</f>
+        <v/>
+      </c>
+      <c r="O23" s="19" t="inlineStr">
         <is>
           <t>สับ PVD+RMF เข้าตราสารหนี้ | บำนาญ 85/5 (ปี 3/5)</t>
         </is>
@@ -1849,25 +1789,22 @@
       <c r="J24" s="6" t="n">
         <v>12500</v>
       </c>
-      <c r="K24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="9">
-        <f>SUM(G24:K24)</f>
-        <v/>
-      </c>
-      <c r="M24" s="6" t="n">
+      <c r="K24" s="9">
+        <f>SUM(G24:J24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="6" t="n">
         <v>100000</v>
       </c>
-      <c r="N24" s="10">
-        <f>L24*12+M24</f>
-        <v/>
-      </c>
-      <c r="O24" s="11">
-        <f>F24-N24</f>
-        <v/>
-      </c>
-      <c r="P24" s="12" t="inlineStr">
+      <c r="M24" s="10">
+        <f>K24*12+L24</f>
+        <v/>
+      </c>
+      <c r="N24" s="11">
+        <f>F24-M24</f>
+        <v/>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
         <is>
           <t>บำนาญ 85/5 (ปี 4/5) | ปรับเบี้ยสุขภาพช่วง 56-60</t>
         </is>
@@ -1904,25 +1841,22 @@
       <c r="J25" s="22" t="n">
         <v>12500</v>
       </c>
-      <c r="K25" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="9">
-        <f>SUM(G25:K25)</f>
-        <v/>
-      </c>
-      <c r="M25" s="22" t="n">
+      <c r="K25" s="9">
+        <f>SUM(G25:J25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="22" t="n">
         <v>100000</v>
       </c>
-      <c r="N25" s="10">
-        <f>L25*12+M25</f>
-        <v/>
-      </c>
-      <c r="O25" s="25">
-        <f>F25-N25</f>
-        <v/>
-      </c>
-      <c r="P25" s="26" t="inlineStr">
+      <c r="M25" s="10">
+        <f>K25*12+L25</f>
+        <v/>
+      </c>
+      <c r="N25" s="25">
+        <f>F25-M25</f>
+        <v/>
+      </c>
+      <c r="O25" s="26" t="inlineStr">
         <is>
           <t>ส่งประกันสะสมทรัพย์งวดสุดท้าย | บำนาญ 85/5 งวดสุดท้าย (ปี 5/5)</t>
         </is>
@@ -1959,25 +1893,22 @@
       <c r="J26" s="6" t="n">
         <v>9167</v>
       </c>
-      <c r="K26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="9">
-        <f>SUM(G26:K26)</f>
-        <v/>
-      </c>
-      <c r="M26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="10">
-        <f>L26*12+M26</f>
-        <v/>
-      </c>
-      <c r="O26" s="11">
-        <f>F26-N26</f>
-        <v/>
-      </c>
-      <c r="P26" s="12" t="inlineStr">
+      <c r="K26" s="9">
+        <f>SUM(G26:J26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="10">
+        <f>K26*12+L26</f>
+        <v/>
+      </c>
+      <c r="N26" s="11">
+        <f>F26-M26</f>
+        <v/>
+      </c>
+      <c r="O26" s="12" t="inlineStr">
         <is>
           <t>หยุดส่งสะสมทรัพย์ (รับเงินคืน 250k เข้า e-Savings) เหลือส่งบำนาญเดิม+สุขภาพ</t>
         </is>
@@ -2014,25 +1945,22 @@
       <c r="J27" s="15" t="n">
         <v>9167</v>
       </c>
-      <c r="K27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="L27" s="9">
-        <f>SUM(G27:K27)</f>
-        <v/>
-      </c>
-      <c r="M27" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="N27" s="10">
-        <f>L27*12+M27</f>
-        <v/>
-      </c>
-      <c r="O27" s="18">
-        <f>F27-N27</f>
-        <v/>
-      </c>
-      <c r="P27" s="19" t="inlineStr">
+      <c r="K27" s="9">
+        <f>SUM(G27:J27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" s="10">
+        <f>K27*12+L27</f>
+        <v/>
+      </c>
+      <c r="N27" s="18">
+        <f>F27-M27</f>
+        <v/>
+      </c>
+      <c r="O27" s="19" t="inlineStr">
         <is>
           <t>เตรียมความพร้อมก่อนเกษียณ 1 ปี (วางแผนโยก PVD เข้า สอ. ภายใน 60 วัน)</t>
         </is>
@@ -2069,25 +1997,22 @@
       <c r="J28" s="22" t="n">
         <v>9167</v>
       </c>
-      <c r="K28" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="9">
-        <f>SUM(G28:K28)</f>
-        <v/>
-      </c>
-      <c r="M28" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="10">
-        <f>L28*12+M28</f>
-        <v/>
-      </c>
-      <c r="O28" s="25">
-        <f>F28-N28</f>
-        <v/>
-      </c>
-      <c r="P28" s="26" t="inlineStr">
+      <c r="K28" s="9">
+        <f>SUM(G28:J28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" s="10">
+        <f>K28*12+L28</f>
+        <v/>
+      </c>
+      <c r="N28" s="25">
+        <f>F28-M28</f>
+        <v/>
+      </c>
+      <c r="O28" s="26" t="inlineStr">
         <is>
           <t>ปีสุดท้าย: ส่งบำนาญเดิมงวดสุดท้าย + รับเงินชดเชยเกษียณ 400 วัน 1.312M + โยก PVD 5M ฝากพิเศษเกษียณสุข</t>
         </is>
@@ -2128,14 +2053,14 @@
         <f>SUM(J6:J28)*12</f>
         <v/>
       </c>
-      <c r="K29" s="29">
-        <f>SUM(K6:K28)*12</f>
-        <v/>
-      </c>
-      <c r="L29" s="28" t="inlineStr">
+      <c r="K29" s="28" t="inlineStr">
         <is>
           <t>-</t>
         </is>
+      </c>
+      <c r="L29" s="29">
+        <f>SUM(L6:L28)</f>
+        <v/>
       </c>
       <c r="M29" s="29">
         <f>SUM(M6:M28)</f>
@@ -2145,11 +2070,7 @@
         <f>SUM(N6:N28)</f>
         <v/>
       </c>
-      <c r="O29" s="29">
-        <f>SUM(O6:O28)</f>
-        <v/>
-      </c>
-      <c r="P29" s="27" t="inlineStr">
+      <c r="O29" s="27" t="inlineStr">
         <is>
           <t>ยอดรวมสะสมตลอด 23 ปี สู่เป้าหมาย 25 ล้านบาท</t>
         </is>

</xml_diff>